<commit_message>
Miyawaki nord-est: luminișul mutat cu cel puțin 6 m de pădure de jur împrejur, aleea în cârlig refăcută; plan, irigare, comenzi și coordonate de trasare regenerate
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017cfyCLE359cmg5Q5QJewA2
</commit_message>
<xml_diff>
--- a/resurse/oferte/cereri/cerere-oferta-pepiniera-silvica-agigea.xlsx
+++ b/resurse/oferte/cereri/cerere-oferta-pepiniera-silvica-agigea.xlsx
@@ -580,7 +580,7 @@
         </is>
       </c>
       <c r="D11" s="5" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
@@ -812,7 +812,7 @@
         </is>
       </c>
       <c r="D19" s="5" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>

</xml_diff>